<commit_message>
Created files to reduce main.py
</commit_message>
<xml_diff>
--- a/Test/Excel test.xlsx
+++ b/Test/Excel test.xlsx
@@ -26,18 +26,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00CCCCCC"/>
-        <bgColor rgb="00CCCCCC"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -64,16 +58,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG7"/>
+  <dimension ref="A1:AG3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -711,224 +704,44 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>12h / 154h</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>12h / 161h</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
-      <c r="O3" s="4" t="inlineStr"/>
-      <c r="P3" s="4" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
-      <c r="V3" s="4" t="inlineStr"/>
-      <c r="W3" s="4" t="inlineStr"/>
+      <c r="V3" s="3" t="inlineStr"/>
+      <c r="W3" s="3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
-      <c r="AC3" s="4" t="inlineStr"/>
-      <c r="AD3" s="4" t="inlineStr"/>
+      <c r="AC3" s="3" t="inlineStr"/>
+      <c r="AD3" s="3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Z. Zerg</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>0h / 154h</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" s="4" t="inlineStr"/>
-      <c r="P4" s="4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" s="4" t="inlineStr"/>
-      <c r="W4" s="4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" s="4" t="inlineStr"/>
-      <c r="AD4" s="4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Z. Gez</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>0h / 154h</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" s="4" t="inlineStr"/>
-      <c r="P5" s="4" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" s="4" t="inlineStr"/>
-      <c r="W5" s="4" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" s="4" t="inlineStr"/>
-      <c r="AD5" s="4" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>R. Zer</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>12h / 154h</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" s="4" t="inlineStr"/>
-      <c r="P6" s="4" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" s="4" t="inlineStr"/>
-      <c r="W6" s="4" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" s="4" t="inlineStr"/>
-      <c r="AD6" s="4" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>E. Aze</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>12h / 154h</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="4" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" s="4" t="inlineStr"/>
-      <c r="W7" s="4" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" s="4" t="inlineStr"/>
-      <c r="AD7" s="4" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
A lot has changed, and everything works !
</commit_message>
<xml_diff>
--- a/Test/Excel test.xlsx
+++ b/Test/Excel test.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DECEMBER 2025" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="JANUARY 2025" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +26,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -37,6 +37,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00DDDDDD"/>
         <bgColor rgb="00DDDDDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ADD8FF"/>
+        <bgColor rgb="00ADD8FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -58,12 +64,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -442,162 +455,162 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DECEMBER 2025</t>
+          <t>JANUARY 2025</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Mer</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Jeu</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ven</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Dim</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Lun</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Mer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Jeu</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Ven</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Sam</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Dim</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Lun</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Mer</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Jeu</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Ven</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>Sam</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>Dim</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Lun</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Mer</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Jeu</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Ven</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>Sam</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>Dim</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Lun</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Mer</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Jeu</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Ven</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Sam</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Dim</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Lun</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Mer</t>
         </is>
       </c>
     </row>
@@ -611,10 +624,10 @@
       <c r="E2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G2" s="2" t="n">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="n">
@@ -632,10 +645,10 @@
       <c r="L2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="M2" s="1" t="n">
+      <c r="M2" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="N2" s="1" t="n">
+      <c r="N2" s="2" t="n">
         <v>12</v>
       </c>
       <c r="O2" s="1" t="n">
@@ -653,10 +666,10 @@
       <c r="S2" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="T2" s="1" t="n">
+      <c r="T2" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="U2" s="1" t="n">
+      <c r="U2" s="2" t="n">
         <v>19</v>
       </c>
       <c r="V2" s="1" t="n">
@@ -674,10 +687,10 @@
       <c r="Z2" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="AA2" s="1" t="n">
+      <c r="AA2" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="AB2" s="1" t="n">
+      <c r="AB2" s="2" t="n">
         <v>26</v>
       </c>
       <c r="AC2" s="1" t="n">
@@ -697,48 +710,48 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>T. Angibaud</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>T. Angibaud  %</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>12h / 161h</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr"/>
+      <c r="M3" s="6" t="inlineStr"/>
+      <c r="N3" s="6" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" s="3" t="inlineStr"/>
-      <c r="W3" s="3" t="inlineStr"/>
+      <c r="T3" s="6" t="inlineStr"/>
+      <c r="U3" s="6" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" s="3" t="inlineStr"/>
-      <c r="AD3" s="3" t="inlineStr"/>
+      <c r="AA3" s="6" t="inlineStr"/>
+      <c r="AB3" s="6" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>

</xml_diff>

<commit_message>
Changed editor, changed everything
</commit_message>
<xml_diff>
--- a/Test/Excel test.xlsx
+++ b/Test/Excel test.xlsx
@@ -26,7 +26,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -41,8 +41,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCCCCC"/>
-        <bgColor rgb="00CCCCCC"/>
+        <fgColor rgb="005555ff"/>
+        <bgColor rgb="005555ff"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000c300"/>
+        <bgColor rgb="0000c300"/>
       </patternFill>
     </fill>
     <fill>
@@ -64,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -73,8 +79,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -719,40 +730,56 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
+      <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" s="6" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
-      <c r="S4" s="5" t="inlineStr"/>
-      <c r="T4" s="5" t="inlineStr"/>
+      <c r="S4" s="6" t="inlineStr"/>
+      <c r="T4" s="6" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
-      <c r="Z4" s="5" t="inlineStr"/>
-      <c r="AA4" s="5" t="inlineStr"/>
+      <c r="Z4" s="6" t="inlineStr"/>
+      <c r="AA4" s="6" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
-      <c r="AG4" s="5" t="inlineStr"/>
+      <c r="AG4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -769,40 +796,40 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr"/>
+      <c r="M6" s="6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" s="5" t="inlineStr"/>
-      <c r="T6" s="5" t="inlineStr"/>
+      <c r="S6" s="6" t="inlineStr"/>
+      <c r="T6" s="6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
-      <c r="Z6" s="5" t="inlineStr"/>
-      <c r="AA6" s="5" t="inlineStr"/>
+      <c r="Z6" s="6" t="inlineStr"/>
+      <c r="AA6" s="6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
-      <c r="AG6" s="5" t="inlineStr"/>
+      <c r="AG6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -812,40 +839,40 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr"/>
-      <c r="M7" s="5" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
-      <c r="S7" s="5" t="inlineStr"/>
-      <c r="T7" s="5" t="inlineStr"/>
+      <c r="S7" s="6" t="inlineStr"/>
+      <c r="T7" s="6" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
-      <c r="Z7" s="5" t="inlineStr"/>
-      <c r="AA7" s="5" t="inlineStr"/>
+      <c r="Z7" s="6" t="inlineStr"/>
+      <c r="AA7" s="6" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
-      <c r="AG7" s="5" t="inlineStr"/>
+      <c r="AG7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -855,40 +882,40 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
+      <c r="M8" s="6" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
-      <c r="S8" s="5" t="inlineStr"/>
-      <c r="T8" s="5" t="inlineStr"/>
+      <c r="S8" s="6" t="inlineStr"/>
+      <c r="T8" s="6" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
-      <c r="Z8" s="5" t="inlineStr"/>
-      <c r="AA8" s="5" t="inlineStr"/>
+      <c r="Z8" s="6" t="inlineStr"/>
+      <c r="AA8" s="6" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
-      <c r="AG8" s="5" t="inlineStr"/>
+      <c r="AG8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -898,40 +925,40 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
+      <c r="D9" s="6" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr"/>
-      <c r="M9" s="5" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
-      <c r="S9" s="5" t="inlineStr"/>
-      <c r="T9" s="5" t="inlineStr"/>
+      <c r="S9" s="6" t="inlineStr"/>
+      <c r="T9" s="6" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
-      <c r="Z9" s="5" t="inlineStr"/>
-      <c r="AA9" s="5" t="inlineStr"/>
+      <c r="Z9" s="6" t="inlineStr"/>
+      <c r="AA9" s="6" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
-      <c r="AG9" s="5" t="inlineStr"/>
+      <c r="AG9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -948,40 +975,40 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="5" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" s="5" t="inlineStr"/>
-      <c r="M11" s="5" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
+      <c r="M11" s="6" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" s="5" t="inlineStr"/>
-      <c r="T11" s="5" t="inlineStr"/>
+      <c r="S11" s="6" t="inlineStr"/>
+      <c r="T11" s="6" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
-      <c r="Z11" s="5" t="inlineStr"/>
-      <c r="AA11" s="5" t="inlineStr"/>
+      <c r="Z11" s="6" t="inlineStr"/>
+      <c r="AA11" s="6" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
-      <c r="AG11" s="5" t="inlineStr"/>
+      <c r="AG11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -991,40 +1018,40 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr"/>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" s="5" t="inlineStr"/>
-      <c r="M12" s="5" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
+      <c r="M12" s="6" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
-      <c r="S12" s="5" t="inlineStr"/>
-      <c r="T12" s="5" t="inlineStr"/>
+      <c r="S12" s="6" t="inlineStr"/>
+      <c r="T12" s="6" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
-      <c r="Z12" s="5" t="inlineStr"/>
-      <c r="AA12" s="5" t="inlineStr"/>
+      <c r="Z12" s="6" t="inlineStr"/>
+      <c r="AA12" s="6" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr"/>
-      <c r="AG12" s="5" t="inlineStr"/>
+      <c r="AG12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1041,40 +1068,40 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="5" t="inlineStr"/>
-      <c r="F14" s="5" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="D14" s="6" t="inlineStr"/>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" s="5" t="inlineStr"/>
-      <c r="M14" s="5" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
+      <c r="M14" s="6" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
-      <c r="S14" s="5" t="inlineStr"/>
-      <c r="T14" s="5" t="inlineStr"/>
+      <c r="S14" s="6" t="inlineStr"/>
+      <c r="T14" s="6" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
-      <c r="Z14" s="5" t="inlineStr"/>
-      <c r="AA14" s="5" t="inlineStr"/>
+      <c r="Z14" s="6" t="inlineStr"/>
+      <c r="AA14" s="6" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr"/>
-      <c r="AG14" s="5" t="inlineStr"/>
+      <c r="AG14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1084,40 +1111,40 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>0h / 109h</t>
+          <t>0h / 116h</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="5" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
+      <c r="D15" s="6" t="inlineStr"/>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" s="5" t="inlineStr"/>
-      <c r="M15" s="5" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr"/>
+      <c r="M15" s="6" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
-      <c r="S15" s="5" t="inlineStr"/>
-      <c r="T15" s="5" t="inlineStr"/>
+      <c r="S15" s="6" t="inlineStr"/>
+      <c r="T15" s="6" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
-      <c r="Z15" s="5" t="inlineStr"/>
-      <c r="AA15" s="5" t="inlineStr"/>
+      <c r="Z15" s="6" t="inlineStr"/>
+      <c r="AA15" s="6" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr"/>
-      <c r="AG15" s="5" t="inlineStr"/>
+      <c r="AG15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1127,40 +1154,40 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr"/>
-      <c r="F16" s="5" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
+      <c r="D16" s="6" t="inlineStr"/>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" s="5" t="inlineStr"/>
-      <c r="M16" s="5" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr"/>
+      <c r="M16" s="6" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
-      <c r="S16" s="5" t="inlineStr"/>
-      <c r="T16" s="5" t="inlineStr"/>
+      <c r="S16" s="6" t="inlineStr"/>
+      <c r="T16" s="6" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
-      <c r="Z16" s="5" t="inlineStr"/>
-      <c r="AA16" s="5" t="inlineStr"/>
+      <c r="Z16" s="6" t="inlineStr"/>
+      <c r="AA16" s="6" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr"/>
-      <c r="AG16" s="5" t="inlineStr"/>
+      <c r="AG16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1170,40 +1197,40 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>0h / 93h</t>
+          <t>0h / 100h</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="5" t="inlineStr"/>
-      <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr"/>
+      <c r="D17" s="6" t="inlineStr"/>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" s="5" t="inlineStr"/>
-      <c r="M17" s="5" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
-      <c r="S17" s="5" t="inlineStr"/>
-      <c r="T17" s="5" t="inlineStr"/>
+      <c r="S17" s="6" t="inlineStr"/>
+      <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
-      <c r="Z17" s="5" t="inlineStr"/>
-      <c r="AA17" s="5" t="inlineStr"/>
+      <c r="Z17" s="6" t="inlineStr"/>
+      <c r="AA17" s="6" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr"/>
-      <c r="AG17" s="5" t="inlineStr"/>
+      <c r="AG17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1213,40 +1240,40 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr"/>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="4" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr"/>
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" s="5" t="inlineStr"/>
-      <c r="M18" s="5" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr"/>
+      <c r="M18" s="6" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
-      <c r="S18" s="5" t="inlineStr"/>
-      <c r="T18" s="5" t="inlineStr"/>
+      <c r="S18" s="6" t="inlineStr"/>
+      <c r="T18" s="6" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
-      <c r="Z18" s="5" t="inlineStr"/>
-      <c r="AA18" s="5" t="inlineStr"/>
+      <c r="Z18" s="6" t="inlineStr"/>
+      <c r="AA18" s="6" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr"/>
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr"/>
-      <c r="AG18" s="5" t="inlineStr"/>
+      <c r="AG18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1256,40 +1283,40 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="5" t="inlineStr"/>
-      <c r="F19" s="5" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr"/>
+      <c r="D19" s="6" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" s="5" t="inlineStr"/>
-      <c r="M19" s="5" t="inlineStr"/>
+      <c r="L19" s="6" t="inlineStr"/>
+      <c r="M19" s="6" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
-      <c r="S19" s="5" t="inlineStr"/>
-      <c r="T19" s="5" t="inlineStr"/>
+      <c r="S19" s="6" t="inlineStr"/>
+      <c r="T19" s="6" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr"/>
-      <c r="Z19" s="5" t="inlineStr"/>
-      <c r="AA19" s="5" t="inlineStr"/>
+      <c r="Z19" s="6" t="inlineStr"/>
+      <c r="AA19" s="6" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr"/>
       <c r="AD19" t="inlineStr"/>
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr"/>
-      <c r="AG19" s="5" t="inlineStr"/>
+      <c r="AG19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1299,40 +1326,40 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>0h / 63h</t>
+          <t>0h / 70h</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr"/>
+      <c r="D20" s="6" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" s="5" t="inlineStr"/>
-      <c r="M20" s="5" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
+      <c r="M20" s="6" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
-      <c r="S20" s="5" t="inlineStr"/>
-      <c r="T20" s="5" t="inlineStr"/>
+      <c r="S20" s="6" t="inlineStr"/>
+      <c r="T20" s="6" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr"/>
-      <c r="Z20" s="5" t="inlineStr"/>
-      <c r="AA20" s="5" t="inlineStr"/>
+      <c r="Z20" s="6" t="inlineStr"/>
+      <c r="AA20" s="6" t="inlineStr"/>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr"/>
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr"/>
-      <c r="AG20" s="5" t="inlineStr"/>
+      <c r="AG20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1349,40 +1376,40 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>0h / 63h</t>
+          <t>0h / 70h</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="5" t="inlineStr"/>
-      <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr"/>
+      <c r="D22" s="6" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" s="5" t="inlineStr"/>
-      <c r="M22" s="5" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr"/>
+      <c r="M22" s="6" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
-      <c r="S22" s="5" t="inlineStr"/>
-      <c r="T22" s="5" t="inlineStr"/>
+      <c r="S22" s="6" t="inlineStr"/>
+      <c r="T22" s="6" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
-      <c r="Z22" s="5" t="inlineStr"/>
-      <c r="AA22" s="5" t="inlineStr"/>
+      <c r="Z22" s="6" t="inlineStr"/>
+      <c r="AA22" s="6" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr"/>
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr"/>
-      <c r="AG22" s="5" t="inlineStr"/>
+      <c r="AG22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1392,40 +1419,40 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>0h / 109h</t>
+          <t>0h / 116h</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr"/>
-      <c r="F23" s="5" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr"/>
+      <c r="D23" s="6" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" s="5" t="inlineStr"/>
-      <c r="M23" s="5" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr"/>
+      <c r="M23" s="6" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
-      <c r="S23" s="5" t="inlineStr"/>
-      <c r="T23" s="5" t="inlineStr"/>
+      <c r="S23" s="6" t="inlineStr"/>
+      <c r="T23" s="6" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="inlineStr"/>
-      <c r="Z23" s="5" t="inlineStr"/>
-      <c r="AA23" s="5" t="inlineStr"/>
+      <c r="Z23" s="6" t="inlineStr"/>
+      <c r="AA23" s="6" t="inlineStr"/>
       <c r="AB23" t="inlineStr"/>
       <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="inlineStr"/>
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr"/>
-      <c r="AG23" s="5" t="inlineStr"/>
+      <c r="AG23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -1442,40 +1469,40 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="5" t="inlineStr"/>
-      <c r="F25" s="5" t="inlineStr"/>
-      <c r="G25" s="4" t="inlineStr"/>
+      <c r="D25" s="6" t="inlineStr"/>
+      <c r="E25" s="6" t="inlineStr"/>
+      <c r="F25" s="6" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" s="5" t="inlineStr"/>
-      <c r="M25" s="5" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr"/>
+      <c r="M25" s="6" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
-      <c r="S25" s="5" t="inlineStr"/>
-      <c r="T25" s="5" t="inlineStr"/>
+      <c r="S25" s="6" t="inlineStr"/>
+      <c r="T25" s="6" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr"/>
-      <c r="Z25" s="5" t="inlineStr"/>
-      <c r="AA25" s="5" t="inlineStr"/>
+      <c r="Z25" s="6" t="inlineStr"/>
+      <c r="AA25" s="6" t="inlineStr"/>
       <c r="AB25" t="inlineStr"/>
       <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="inlineStr"/>
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr"/>
-      <c r="AG25" s="5" t="inlineStr"/>
+      <c r="AG25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1485,40 +1512,40 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>0h / 63h</t>
+          <t>0h / 70h</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="5" t="inlineStr"/>
-      <c r="F26" s="5" t="inlineStr"/>
-      <c r="G26" s="4" t="inlineStr"/>
+      <c r="D26" s="6" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr"/>
+      <c r="F26" s="6" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" s="5" t="inlineStr"/>
-      <c r="M26" s="5" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr"/>
+      <c r="M26" s="6" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
-      <c r="S26" s="5" t="inlineStr"/>
-      <c r="T26" s="5" t="inlineStr"/>
+      <c r="S26" s="6" t="inlineStr"/>
+      <c r="T26" s="6" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr"/>
-      <c r="Z26" s="5" t="inlineStr"/>
-      <c r="AA26" s="5" t="inlineStr"/>
+      <c r="Z26" s="6" t="inlineStr"/>
+      <c r="AA26" s="6" t="inlineStr"/>
       <c r="AB26" t="inlineStr"/>
       <c r="AC26" t="inlineStr"/>
       <c r="AD26" t="inlineStr"/>
       <c r="AE26" t="inlineStr"/>
       <c r="AF26" t="inlineStr"/>
-      <c r="AG26" s="5" t="inlineStr"/>
+      <c r="AG26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1528,40 +1555,40 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="5" t="inlineStr"/>
-      <c r="F27" s="5" t="inlineStr"/>
-      <c r="G27" s="4" t="inlineStr"/>
+      <c r="D27" s="6" t="inlineStr"/>
+      <c r="E27" s="6" t="inlineStr"/>
+      <c r="F27" s="6" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" s="5" t="inlineStr"/>
-      <c r="M27" s="5" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr"/>
+      <c r="M27" s="6" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
-      <c r="S27" s="5" t="inlineStr"/>
-      <c r="T27" s="5" t="inlineStr"/>
+      <c r="S27" s="6" t="inlineStr"/>
+      <c r="T27" s="6" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="inlineStr"/>
-      <c r="Z27" s="5" t="inlineStr"/>
-      <c r="AA27" s="5" t="inlineStr"/>
+      <c r="Z27" s="6" t="inlineStr"/>
+      <c r="AA27" s="6" t="inlineStr"/>
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="inlineStr"/>
       <c r="AD27" t="inlineStr"/>
       <c r="AE27" t="inlineStr"/>
       <c r="AF27" t="inlineStr"/>
-      <c r="AG27" s="5" t="inlineStr"/>
+      <c r="AG27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1571,40 +1598,40 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="5" t="inlineStr"/>
-      <c r="F28" s="5" t="inlineStr"/>
-      <c r="G28" s="4" t="inlineStr"/>
+      <c r="D28" s="6" t="inlineStr"/>
+      <c r="E28" s="6" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" s="5" t="inlineStr"/>
-      <c r="M28" s="5" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr"/>
+      <c r="M28" s="6" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
-      <c r="S28" s="5" t="inlineStr"/>
-      <c r="T28" s="5" t="inlineStr"/>
+      <c r="S28" s="6" t="inlineStr"/>
+      <c r="T28" s="6" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
-      <c r="Z28" s="5" t="inlineStr"/>
-      <c r="AA28" s="5" t="inlineStr"/>
+      <c r="Z28" s="6" t="inlineStr"/>
+      <c r="AA28" s="6" t="inlineStr"/>
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="inlineStr"/>
       <c r="AD28" t="inlineStr"/>
       <c r="AE28" t="inlineStr"/>
       <c r="AF28" t="inlineStr"/>
-      <c r="AG28" s="5" t="inlineStr"/>
+      <c r="AG28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -1621,40 +1648,40 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr"/>
-      <c r="E30" s="5" t="inlineStr"/>
-      <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="4" t="inlineStr"/>
+      <c r="D30" s="6" t="inlineStr"/>
+      <c r="E30" s="6" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" s="5" t="inlineStr"/>
-      <c r="M30" s="5" t="inlineStr"/>
+      <c r="L30" s="6" t="inlineStr"/>
+      <c r="M30" s="6" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
-      <c r="S30" s="5" t="inlineStr"/>
-      <c r="T30" s="5" t="inlineStr"/>
+      <c r="S30" s="6" t="inlineStr"/>
+      <c r="T30" s="6" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
-      <c r="Z30" s="5" t="inlineStr"/>
-      <c r="AA30" s="5" t="inlineStr"/>
+      <c r="Z30" s="6" t="inlineStr"/>
+      <c r="AA30" s="6" t="inlineStr"/>
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="inlineStr"/>
       <c r="AD30" t="inlineStr"/>
       <c r="AE30" t="inlineStr"/>
       <c r="AF30" t="inlineStr"/>
-      <c r="AG30" s="5" t="inlineStr"/>
+      <c r="AG30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1664,40 +1691,40 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr"/>
-      <c r="E31" s="5" t="inlineStr"/>
-      <c r="F31" s="5" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr"/>
+      <c r="D31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr"/>
+      <c r="F31" s="6" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" s="5" t="inlineStr"/>
-      <c r="M31" s="5" t="inlineStr"/>
+      <c r="L31" s="6" t="inlineStr"/>
+      <c r="M31" s="6" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
-      <c r="S31" s="5" t="inlineStr"/>
-      <c r="T31" s="5" t="inlineStr"/>
+      <c r="S31" s="6" t="inlineStr"/>
+      <c r="T31" s="6" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
       <c r="Y31" t="inlineStr"/>
-      <c r="Z31" s="5" t="inlineStr"/>
-      <c r="AA31" s="5" t="inlineStr"/>
+      <c r="Z31" s="6" t="inlineStr"/>
+      <c r="AA31" s="6" t="inlineStr"/>
       <c r="AB31" t="inlineStr"/>
       <c r="AC31" t="inlineStr"/>
       <c r="AD31" t="inlineStr"/>
       <c r="AE31" t="inlineStr"/>
       <c r="AF31" t="inlineStr"/>
-      <c r="AG31" s="5" t="inlineStr"/>
+      <c r="AG31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1707,40 +1734,40 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="5" t="inlineStr"/>
-      <c r="F32" s="5" t="inlineStr"/>
-      <c r="G32" s="4" t="inlineStr"/>
+      <c r="D32" s="6" t="inlineStr"/>
+      <c r="E32" s="6" t="inlineStr"/>
+      <c r="F32" s="6" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" s="5" t="inlineStr"/>
-      <c r="M32" s="5" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr"/>
+      <c r="M32" s="6" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
-      <c r="S32" s="5" t="inlineStr"/>
-      <c r="T32" s="5" t="inlineStr"/>
+      <c r="S32" s="6" t="inlineStr"/>
+      <c r="T32" s="6" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
       <c r="Y32" t="inlineStr"/>
-      <c r="Z32" s="5" t="inlineStr"/>
-      <c r="AA32" s="5" t="inlineStr"/>
+      <c r="Z32" s="6" t="inlineStr"/>
+      <c r="AA32" s="6" t="inlineStr"/>
       <c r="AB32" t="inlineStr"/>
       <c r="AC32" t="inlineStr"/>
       <c r="AD32" t="inlineStr"/>
       <c r="AE32" t="inlineStr"/>
       <c r="AF32" t="inlineStr"/>
-      <c r="AG32" s="5" t="inlineStr"/>
+      <c r="AG32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1750,40 +1777,40 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>0h / 63h</t>
+          <t>0h / 70h</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="5" t="inlineStr"/>
-      <c r="F33" s="5" t="inlineStr"/>
-      <c r="G33" s="4" t="inlineStr"/>
+      <c r="D33" s="6" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr"/>
+      <c r="F33" s="6" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" s="5" t="inlineStr"/>
-      <c r="M33" s="5" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr"/>
+      <c r="M33" s="6" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
-      <c r="S33" s="5" t="inlineStr"/>
-      <c r="T33" s="5" t="inlineStr"/>
+      <c r="S33" s="6" t="inlineStr"/>
+      <c r="T33" s="6" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
       <c r="X33" t="inlineStr"/>
       <c r="Y33" t="inlineStr"/>
-      <c r="Z33" s="5" t="inlineStr"/>
-      <c r="AA33" s="5" t="inlineStr"/>
+      <c r="Z33" s="6" t="inlineStr"/>
+      <c r="AA33" s="6" t="inlineStr"/>
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr"/>
       <c r="AD33" t="inlineStr"/>
       <c r="AE33" t="inlineStr"/>
       <c r="AF33" t="inlineStr"/>
-      <c r="AG33" s="5" t="inlineStr"/>
+      <c r="AG33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1793,40 +1820,40 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr"/>
-      <c r="E34" s="5" t="inlineStr"/>
-      <c r="F34" s="5" t="inlineStr"/>
-      <c r="G34" s="4" t="inlineStr"/>
+      <c r="D34" s="6" t="inlineStr"/>
+      <c r="E34" s="6" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" s="5" t="inlineStr"/>
-      <c r="M34" s="5" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr"/>
+      <c r="M34" s="6" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
-      <c r="S34" s="5" t="inlineStr"/>
-      <c r="T34" s="5" t="inlineStr"/>
+      <c r="S34" s="6" t="inlineStr"/>
+      <c r="T34" s="6" t="inlineStr"/>
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr"/>
       <c r="W34" t="inlineStr"/>
       <c r="X34" t="inlineStr"/>
       <c r="Y34" t="inlineStr"/>
-      <c r="Z34" s="5" t="inlineStr"/>
-      <c r="AA34" s="5" t="inlineStr"/>
+      <c r="Z34" s="6" t="inlineStr"/>
+      <c r="AA34" s="6" t="inlineStr"/>
       <c r="AB34" t="inlineStr"/>
       <c r="AC34" t="inlineStr"/>
       <c r="AD34" t="inlineStr"/>
       <c r="AE34" t="inlineStr"/>
       <c r="AF34" t="inlineStr"/>
-      <c r="AG34" s="5" t="inlineStr"/>
+      <c r="AG34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1836,40 +1863,40 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>0h / 63h</t>
+          <t>0h / 70h</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="5" t="inlineStr"/>
-      <c r="F35" s="5" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
+      <c r="D35" s="6" t="inlineStr"/>
+      <c r="E35" s="6" t="inlineStr"/>
+      <c r="F35" s="6" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" s="5" t="inlineStr"/>
-      <c r="M35" s="5" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr"/>
+      <c r="M35" s="6" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
-      <c r="S35" s="5" t="inlineStr"/>
-      <c r="T35" s="5" t="inlineStr"/>
+      <c r="S35" s="6" t="inlineStr"/>
+      <c r="T35" s="6" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr"/>
       <c r="W35" t="inlineStr"/>
       <c r="X35" t="inlineStr"/>
       <c r="Y35" t="inlineStr"/>
-      <c r="Z35" s="5" t="inlineStr"/>
-      <c r="AA35" s="5" t="inlineStr"/>
+      <c r="Z35" s="6" t="inlineStr"/>
+      <c r="AA35" s="6" t="inlineStr"/>
       <c r="AB35" t="inlineStr"/>
       <c r="AC35" t="inlineStr"/>
       <c r="AD35" t="inlineStr"/>
       <c r="AE35" t="inlineStr"/>
       <c r="AF35" t="inlineStr"/>
-      <c r="AG35" s="5" t="inlineStr"/>
+      <c r="AG35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1879,40 +1906,40 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" s="4" t="inlineStr"/>
-      <c r="E36" s="5" t="inlineStr"/>
-      <c r="F36" s="5" t="inlineStr"/>
-      <c r="G36" s="4" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" s="5" t="inlineStr"/>
-      <c r="M36" s="5" t="inlineStr"/>
+      <c r="L36" s="6" t="inlineStr"/>
+      <c r="M36" s="6" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
-      <c r="S36" s="5" t="inlineStr"/>
-      <c r="T36" s="5" t="inlineStr"/>
+      <c r="S36" s="6" t="inlineStr"/>
+      <c r="T36" s="6" t="inlineStr"/>
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr"/>
-      <c r="Z36" s="5" t="inlineStr"/>
-      <c r="AA36" s="5" t="inlineStr"/>
+      <c r="Z36" s="6" t="inlineStr"/>
+      <c r="AA36" s="6" t="inlineStr"/>
       <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="inlineStr"/>
       <c r="AD36" t="inlineStr"/>
       <c r="AE36" t="inlineStr"/>
       <c r="AF36" t="inlineStr"/>
-      <c r="AG36" s="5" t="inlineStr"/>
+      <c r="AG36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1922,40 +1949,40 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>0h / 109h</t>
+          <t>0h / 116h</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="5" t="inlineStr"/>
-      <c r="F37" s="5" t="inlineStr"/>
-      <c r="G37" s="4" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" s="5" t="inlineStr"/>
-      <c r="M37" s="5" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr"/>
+      <c r="M37" s="6" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
-      <c r="S37" s="5" t="inlineStr"/>
-      <c r="T37" s="5" t="inlineStr"/>
+      <c r="S37" s="6" t="inlineStr"/>
+      <c r="T37" s="6" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr"/>
       <c r="Y37" t="inlineStr"/>
-      <c r="Z37" s="5" t="inlineStr"/>
-      <c r="AA37" s="5" t="inlineStr"/>
+      <c r="Z37" s="6" t="inlineStr"/>
+      <c r="AA37" s="6" t="inlineStr"/>
       <c r="AB37" t="inlineStr"/>
       <c r="AC37" t="inlineStr"/>
       <c r="AD37" t="inlineStr"/>
       <c r="AE37" t="inlineStr"/>
       <c r="AF37" t="inlineStr"/>
-      <c r="AG37" s="5" t="inlineStr"/>
+      <c r="AG37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1965,40 +1992,40 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" s="4" t="inlineStr"/>
-      <c r="E38" s="5" t="inlineStr"/>
-      <c r="F38" s="5" t="inlineStr"/>
-      <c r="G38" s="4" t="inlineStr"/>
+      <c r="D38" s="6" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" s="5" t="inlineStr"/>
-      <c r="M38" s="5" t="inlineStr"/>
+      <c r="L38" s="6" t="inlineStr"/>
+      <c r="M38" s="6" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
-      <c r="S38" s="5" t="inlineStr"/>
-      <c r="T38" s="5" t="inlineStr"/>
+      <c r="S38" s="6" t="inlineStr"/>
+      <c r="T38" s="6" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr"/>
       <c r="Y38" t="inlineStr"/>
-      <c r="Z38" s="5" t="inlineStr"/>
-      <c r="AA38" s="5" t="inlineStr"/>
+      <c r="Z38" s="6" t="inlineStr"/>
+      <c r="AA38" s="6" t="inlineStr"/>
       <c r="AB38" t="inlineStr"/>
       <c r="AC38" t="inlineStr"/>
       <c r="AD38" t="inlineStr"/>
       <c r="AE38" t="inlineStr"/>
       <c r="AF38" t="inlineStr"/>
-      <c r="AG38" s="5" t="inlineStr"/>
+      <c r="AG38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2008,40 +2035,40 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" s="4" t="inlineStr"/>
-      <c r="E39" s="5" t="inlineStr"/>
-      <c r="F39" s="5" t="inlineStr"/>
-      <c r="G39" s="4" t="inlineStr"/>
+      <c r="D39" s="6" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" s="5" t="inlineStr"/>
-      <c r="M39" s="5" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr"/>
+      <c r="M39" s="6" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
-      <c r="S39" s="5" t="inlineStr"/>
-      <c r="T39" s="5" t="inlineStr"/>
+      <c r="S39" s="6" t="inlineStr"/>
+      <c r="T39" s="6" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="inlineStr"/>
-      <c r="Z39" s="5" t="inlineStr"/>
-      <c r="AA39" s="5" t="inlineStr"/>
+      <c r="Z39" s="6" t="inlineStr"/>
+      <c r="AA39" s="6" t="inlineStr"/>
       <c r="AB39" t="inlineStr"/>
       <c r="AC39" t="inlineStr"/>
       <c r="AD39" t="inlineStr"/>
       <c r="AE39" t="inlineStr"/>
       <c r="AF39" t="inlineStr"/>
-      <c r="AG39" s="5" t="inlineStr"/>
+      <c r="AG39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2051,40 +2078,40 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr"/>
-      <c r="E40" s="5" t="inlineStr"/>
-      <c r="F40" s="5" t="inlineStr"/>
-      <c r="G40" s="4" t="inlineStr"/>
+      <c r="D40" s="6" t="inlineStr"/>
+      <c r="E40" s="6" t="inlineStr"/>
+      <c r="F40" s="6" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" s="5" t="inlineStr"/>
-      <c r="M40" s="5" t="inlineStr"/>
+      <c r="L40" s="6" t="inlineStr"/>
+      <c r="M40" s="6" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
-      <c r="S40" s="5" t="inlineStr"/>
-      <c r="T40" s="5" t="inlineStr"/>
+      <c r="S40" s="6" t="inlineStr"/>
+      <c r="T40" s="6" t="inlineStr"/>
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr"/>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr"/>
-      <c r="Z40" s="5" t="inlineStr"/>
-      <c r="AA40" s="5" t="inlineStr"/>
+      <c r="Z40" s="6" t="inlineStr"/>
+      <c r="AA40" s="6" t="inlineStr"/>
       <c r="AB40" t="inlineStr"/>
       <c r="AC40" t="inlineStr"/>
       <c r="AD40" t="inlineStr"/>
       <c r="AE40" t="inlineStr"/>
       <c r="AF40" t="inlineStr"/>
-      <c r="AG40" s="5" t="inlineStr"/>
+      <c r="AG40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2094,40 +2121,40 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>0h / 63h</t>
+          <t>0h / 70h</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr"/>
-      <c r="E41" s="5" t="inlineStr"/>
-      <c r="F41" s="5" t="inlineStr"/>
-      <c r="G41" s="4" t="inlineStr"/>
+      <c r="D41" s="6" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" s="5" t="inlineStr"/>
-      <c r="M41" s="5" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr"/>
+      <c r="M41" s="6" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
-      <c r="S41" s="5" t="inlineStr"/>
-      <c r="T41" s="5" t="inlineStr"/>
+      <c r="S41" s="6" t="inlineStr"/>
+      <c r="T41" s="6" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr"/>
       <c r="X41" t="inlineStr"/>
       <c r="Y41" t="inlineStr"/>
-      <c r="Z41" s="5" t="inlineStr"/>
-      <c r="AA41" s="5" t="inlineStr"/>
+      <c r="Z41" s="6" t="inlineStr"/>
+      <c r="AA41" s="6" t="inlineStr"/>
       <c r="AB41" t="inlineStr"/>
       <c r="AC41" t="inlineStr"/>
       <c r="AD41" t="inlineStr"/>
       <c r="AE41" t="inlineStr"/>
       <c r="AF41" t="inlineStr"/>
-      <c r="AG41" s="5" t="inlineStr"/>
+      <c r="AG41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2137,40 +2164,40 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" s="4" t="inlineStr"/>
-      <c r="E42" s="5" t="inlineStr"/>
-      <c r="F42" s="5" t="inlineStr"/>
-      <c r="G42" s="4" t="inlineStr"/>
+      <c r="D42" s="6" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr"/>
+      <c r="F42" s="6" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" s="5" t="inlineStr"/>
-      <c r="M42" s="5" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr"/>
+      <c r="M42" s="6" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
-      <c r="S42" s="5" t="inlineStr"/>
-      <c r="T42" s="5" t="inlineStr"/>
+      <c r="S42" s="6" t="inlineStr"/>
+      <c r="T42" s="6" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="inlineStr"/>
       <c r="Y42" t="inlineStr"/>
-      <c r="Z42" s="5" t="inlineStr"/>
-      <c r="AA42" s="5" t="inlineStr"/>
+      <c r="Z42" s="6" t="inlineStr"/>
+      <c r="AA42" s="6" t="inlineStr"/>
       <c r="AB42" t="inlineStr"/>
       <c r="AC42" t="inlineStr"/>
       <c r="AD42" t="inlineStr"/>
       <c r="AE42" t="inlineStr"/>
       <c r="AF42" t="inlineStr"/>
-      <c r="AG42" s="5" t="inlineStr"/>
+      <c r="AG42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2180,40 +2207,40 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
-      <c r="D43" s="4" t="inlineStr"/>
-      <c r="E43" s="5" t="inlineStr"/>
-      <c r="F43" s="5" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
+      <c r="D43" s="6" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr"/>
+      <c r="F43" s="6" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" s="5" t="inlineStr"/>
-      <c r="M43" s="5" t="inlineStr"/>
+      <c r="L43" s="6" t="inlineStr"/>
+      <c r="M43" s="6" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
-      <c r="S43" s="5" t="inlineStr"/>
-      <c r="T43" s="5" t="inlineStr"/>
+      <c r="S43" s="6" t="inlineStr"/>
+      <c r="T43" s="6" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr"/>
-      <c r="Z43" s="5" t="inlineStr"/>
-      <c r="AA43" s="5" t="inlineStr"/>
+      <c r="Z43" s="6" t="inlineStr"/>
+      <c r="AA43" s="6" t="inlineStr"/>
       <c r="AB43" t="inlineStr"/>
       <c r="AC43" t="inlineStr"/>
       <c r="AD43" t="inlineStr"/>
       <c r="AE43" t="inlineStr"/>
       <c r="AF43" t="inlineStr"/>
-      <c r="AG43" s="5" t="inlineStr"/>
+      <c r="AG43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2223,40 +2250,40 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="5" t="inlineStr"/>
-      <c r="F44" s="5" t="inlineStr"/>
-      <c r="G44" s="4" t="inlineStr"/>
+      <c r="D44" s="6" t="inlineStr"/>
+      <c r="E44" s="6" t="inlineStr"/>
+      <c r="F44" s="6" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" s="5" t="inlineStr"/>
-      <c r="M44" s="5" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr"/>
+      <c r="M44" s="6" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr"/>
-      <c r="S44" s="5" t="inlineStr"/>
-      <c r="T44" s="5" t="inlineStr"/>
+      <c r="S44" s="6" t="inlineStr"/>
+      <c r="T44" s="6" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="inlineStr"/>
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="inlineStr"/>
-      <c r="Z44" s="5" t="inlineStr"/>
-      <c r="AA44" s="5" t="inlineStr"/>
+      <c r="Z44" s="6" t="inlineStr"/>
+      <c r="AA44" s="6" t="inlineStr"/>
       <c r="AB44" t="inlineStr"/>
       <c r="AC44" t="inlineStr"/>
       <c r="AD44" t="inlineStr"/>
       <c r="AE44" t="inlineStr"/>
       <c r="AF44" t="inlineStr"/>
-      <c r="AG44" s="5" t="inlineStr"/>
+      <c r="AG44" s="6" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2266,40 +2293,40 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr"/>
-      <c r="E45" s="5" t="inlineStr"/>
-      <c r="F45" s="5" t="inlineStr"/>
-      <c r="G45" s="4" t="inlineStr"/>
+      <c r="D45" s="6" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" s="5" t="inlineStr"/>
-      <c r="M45" s="5" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr"/>
+      <c r="M45" s="6" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
-      <c r="S45" s="5" t="inlineStr"/>
-      <c r="T45" s="5" t="inlineStr"/>
+      <c r="S45" s="6" t="inlineStr"/>
+      <c r="T45" s="6" t="inlineStr"/>
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr"/>
       <c r="W45" t="inlineStr"/>
       <c r="X45" t="inlineStr"/>
       <c r="Y45" t="inlineStr"/>
-      <c r="Z45" s="5" t="inlineStr"/>
-      <c r="AA45" s="5" t="inlineStr"/>
+      <c r="Z45" s="6" t="inlineStr"/>
+      <c r="AA45" s="6" t="inlineStr"/>
       <c r="AB45" t="inlineStr"/>
       <c r="AC45" t="inlineStr"/>
       <c r="AD45" t="inlineStr"/>
       <c r="AE45" t="inlineStr"/>
       <c r="AF45" t="inlineStr"/>
-      <c r="AG45" s="5" t="inlineStr"/>
+      <c r="AG45" s="6" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2309,40 +2336,40 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
-      <c r="D46" s="4" t="inlineStr"/>
-      <c r="E46" s="5" t="inlineStr"/>
-      <c r="F46" s="5" t="inlineStr"/>
-      <c r="G46" s="4" t="inlineStr"/>
+      <c r="D46" s="6" t="inlineStr"/>
+      <c r="E46" s="6" t="inlineStr"/>
+      <c r="F46" s="6" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" s="5" t="inlineStr"/>
-      <c r="M46" s="5" t="inlineStr"/>
+      <c r="L46" s="6" t="inlineStr"/>
+      <c r="M46" s="6" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
-      <c r="S46" s="5" t="inlineStr"/>
-      <c r="T46" s="5" t="inlineStr"/>
+      <c r="S46" s="6" t="inlineStr"/>
+      <c r="T46" s="6" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr"/>
       <c r="W46" t="inlineStr"/>
       <c r="X46" t="inlineStr"/>
       <c r="Y46" t="inlineStr"/>
-      <c r="Z46" s="5" t="inlineStr"/>
-      <c r="AA46" s="5" t="inlineStr"/>
+      <c r="Z46" s="6" t="inlineStr"/>
+      <c r="AA46" s="6" t="inlineStr"/>
       <c r="AB46" t="inlineStr"/>
       <c r="AC46" t="inlineStr"/>
       <c r="AD46" t="inlineStr"/>
       <c r="AE46" t="inlineStr"/>
       <c r="AF46" t="inlineStr"/>
-      <c r="AG46" s="5" t="inlineStr"/>
+      <c r="AG46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2352,40 +2379,40 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
-      <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="5" t="inlineStr"/>
-      <c r="F47" s="5" t="inlineStr"/>
-      <c r="G47" s="4" t="inlineStr"/>
+      <c r="D47" s="6" t="inlineStr"/>
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" s="5" t="inlineStr"/>
-      <c r="M47" s="5" t="inlineStr"/>
+      <c r="L47" s="6" t="inlineStr"/>
+      <c r="M47" s="6" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
-      <c r="S47" s="5" t="inlineStr"/>
-      <c r="T47" s="5" t="inlineStr"/>
+      <c r="S47" s="6" t="inlineStr"/>
+      <c r="T47" s="6" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="inlineStr"/>
       <c r="X47" t="inlineStr"/>
       <c r="Y47" t="inlineStr"/>
-      <c r="Z47" s="5" t="inlineStr"/>
-      <c r="AA47" s="5" t="inlineStr"/>
+      <c r="Z47" s="6" t="inlineStr"/>
+      <c r="AA47" s="6" t="inlineStr"/>
       <c r="AB47" t="inlineStr"/>
       <c r="AC47" t="inlineStr"/>
       <c r="AD47" t="inlineStr"/>
       <c r="AE47" t="inlineStr"/>
       <c r="AF47" t="inlineStr"/>
-      <c r="AG47" s="5" t="inlineStr"/>
+      <c r="AG47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2395,40 +2422,40 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr"/>
-      <c r="E48" s="5" t="inlineStr"/>
-      <c r="F48" s="5" t="inlineStr"/>
-      <c r="G48" s="4" t="inlineStr"/>
+      <c r="D48" s="6" t="inlineStr"/>
+      <c r="E48" s="6" t="inlineStr"/>
+      <c r="F48" s="6" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" s="5" t="inlineStr"/>
-      <c r="M48" s="5" t="inlineStr"/>
+      <c r="L48" s="6" t="inlineStr"/>
+      <c r="M48" s="6" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
-      <c r="S48" s="5" t="inlineStr"/>
-      <c r="T48" s="5" t="inlineStr"/>
+      <c r="S48" s="6" t="inlineStr"/>
+      <c r="T48" s="6" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr"/>
       <c r="W48" t="inlineStr"/>
       <c r="X48" t="inlineStr"/>
       <c r="Y48" t="inlineStr"/>
-      <c r="Z48" s="5" t="inlineStr"/>
-      <c r="AA48" s="5" t="inlineStr"/>
+      <c r="Z48" s="6" t="inlineStr"/>
+      <c r="AA48" s="6" t="inlineStr"/>
       <c r="AB48" t="inlineStr"/>
       <c r="AC48" t="inlineStr"/>
       <c r="AD48" t="inlineStr"/>
       <c r="AE48" t="inlineStr"/>
       <c r="AF48" t="inlineStr"/>
-      <c r="AG48" s="5" t="inlineStr"/>
+      <c r="AG48" s="6" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
@@ -2445,40 +2472,40 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>0h / 140h</t>
+          <t>0h / 147h</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
-      <c r="D50" s="4" t="inlineStr"/>
-      <c r="E50" s="5" t="inlineStr"/>
-      <c r="F50" s="5" t="inlineStr"/>
-      <c r="G50" s="4" t="inlineStr"/>
+      <c r="D50" s="6" t="inlineStr"/>
+      <c r="E50" s="6" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" s="5" t="inlineStr"/>
-      <c r="M50" s="5" t="inlineStr"/>
+      <c r="L50" s="6" t="inlineStr"/>
+      <c r="M50" s="6" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
-      <c r="S50" s="5" t="inlineStr"/>
-      <c r="T50" s="5" t="inlineStr"/>
+      <c r="S50" s="6" t="inlineStr"/>
+      <c r="T50" s="6" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr"/>
       <c r="W50" t="inlineStr"/>
       <c r="X50" t="inlineStr"/>
       <c r="Y50" t="inlineStr"/>
-      <c r="Z50" s="5" t="inlineStr"/>
-      <c r="AA50" s="5" t="inlineStr"/>
+      <c r="Z50" s="6" t="inlineStr"/>
+      <c r="AA50" s="6" t="inlineStr"/>
       <c r="AB50" t="inlineStr"/>
       <c r="AC50" t="inlineStr"/>
       <c r="AD50" t="inlineStr"/>
       <c r="AE50" t="inlineStr"/>
       <c r="AF50" t="inlineStr"/>
-      <c r="AG50" s="5" t="inlineStr"/>
+      <c r="AG50" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="17">

</xml_diff>